<commit_message>
El material de la CSO siembra 80 señales, más de las 73 que pide un piso del 95 % sin fallas: a la siembra se suma un lote por entidad con las señales que se repiten, cada una en su oportunidad, su cotización o su contrato, sin mover el pronóstico, la meta ni las comisiones; el motor levanta las 80 y ninguna de más
</commit_message>
<xml_diff>
--- a/tests/criterio-cso/material/servicios-mx/comercial/SPM140708QJ2-servicios-profesionales-mexicanos/10-crm/oportunidades-2026-10-01.xlsx
+++ b/tests/criterio-cso/material/servicios-mx/comercial/SPM140708QJ2-servicios-profesionales-mexicanos/10-crm/oportunidades-2026-10-01.xlsx
@@ -433,6 +433,664 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OPP-1520</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pedido marco 20</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CL-1506</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>720000</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>12/12/2026</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OPP-1521</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pedido marco 21</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CL-1500</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>810000</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>12/12/2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OPP-1522</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pedido marco 22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CL-1501</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Negociación</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>900000</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>12/12/2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OPP-1523</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Prospecto 23</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CL-1502</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>720000</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>18/12/2026</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OPP-1524</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Prospecto 24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CL-1503</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>450000</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>18/12/2026</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OPP-1525</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Prospecto 25</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CL-1504</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>540000</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>18/12/2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OPP-1526</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Licencias adicionales 26</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CL-1505</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>720000</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>20/11/2026</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OPP-1527</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Licencias adicionales 27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CL-1506</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>540000</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>20/11/2026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OPP-1528</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Licencias adicionales 28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CL-1500</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>630000</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>20/11/2026</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Fernando Ruiz</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>OPP-1529</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cotización especial 29</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CL-1501</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>900000</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>OPP-1530</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cotización especial 30</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CL-1502</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>990000</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Daniela Ochoa</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>OPP-1531</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Venta directa 31</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CL-1507</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>270000</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Alberto Cano</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>OPP-1532</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Venta directa 32</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CL-1508</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>360000</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Alberto Cano</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OPP-1533</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Venta directa 33</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CL-1509</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Compromiso</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>450000</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Alberto Cano</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>